<commit_message>
inventory matris and etl improvment
</commit_message>
<xml_diff>
--- a/backend/uploads/test_0.xlsx
+++ b/backend/uploads/test_0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BEHNOOD\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8AE30908-9203-4944-931B-C5032490BFC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DF80C60-1F4C-4CBE-827F-8CB9B2CEA23B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{292144CF-731A-4CEA-8ED5-BD45804BE030}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="207">
   <si>
     <t>CAS Number</t>
   </si>
@@ -1488,7 +1488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{144724F1-008E-4839-A1B0-7F8DEE7A437A}">
-  <dimension ref="A3:I54"/>
+  <dimension ref="A3:I56"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.54296875" bestFit="1" customWidth="1"/>
@@ -1981,92 +1981,95 @@
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>204</v>
+      </c>
       <c r="B26" t="s">
-        <v>92</v>
-      </c>
-      <c r="C26">
-        <v>1490</v>
+        <v>0</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1</v>
       </c>
       <c r="D26" t="s">
-        <v>93</v>
+        <v>2</v>
       </c>
       <c r="E26" t="s">
-        <v>94</v>
+        <v>3</v>
       </c>
       <c r="F26" t="s">
-        <v>89</v>
+        <v>4</v>
       </c>
       <c r="G26" t="s">
-        <v>95</v>
-      </c>
-      <c r="H26" s="1">
-        <v>45928</v>
+        <v>5</v>
+      </c>
+      <c r="H26" t="s">
+        <v>6</v>
       </c>
       <c r="I26" t="s">
-        <v>47</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C27">
-        <v>1791</v>
+        <v>1490</v>
       </c>
       <c r="D27" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E27" t="s">
-        <v>35</v>
+        <v>94</v>
       </c>
       <c r="F27" t="s">
         <v>89</v>
       </c>
       <c r="G27" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H27" s="1">
-        <v>46016</v>
+        <v>45928</v>
+      </c>
+      <c r="I27" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C28">
-        <v>1208</v>
+        <v>1791</v>
       </c>
       <c r="D28" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E28" t="s">
         <v>35</v>
       </c>
       <c r="F28" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="G28" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="H28" s="1">
-        <v>45992</v>
-      </c>
-      <c r="I28" t="s">
-        <v>103</v>
+        <v>46016</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B29" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C29">
-        <v>1206</v>
+        <v>1208</v>
       </c>
       <c r="D29" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="E29" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F29" t="s">
         <v>101</v>
@@ -2075,226 +2078,226 @@
         <v>102</v>
       </c>
       <c r="H29" s="1">
-        <v>46034</v>
+        <v>45992</v>
+      </c>
+      <c r="I29" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B30" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C30">
-        <v>1145</v>
+        <v>1206</v>
       </c>
       <c r="D30" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E30" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F30" t="s">
         <v>101</v>
       </c>
       <c r="G30" t="s">
+        <v>102</v>
+      </c>
+      <c r="H30" s="1">
+        <v>46034</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B31" t="s">
+        <v>106</v>
+      </c>
+      <c r="C31">
+        <v>1145</v>
+      </c>
+      <c r="D31" t="s">
+        <v>107</v>
+      </c>
+      <c r="E31" t="s">
+        <v>17</v>
+      </c>
+      <c r="F31" t="s">
+        <v>101</v>
+      </c>
+      <c r="G31" t="s">
         <v>108</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H31" s="1">
         <v>46044</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>109</v>
-      </c>
-      <c r="B31" t="s">
-        <v>110</v>
-      </c>
-      <c r="C31">
-        <v>1155</v>
-      </c>
-      <c r="D31" t="s">
-        <v>111</v>
-      </c>
-      <c r="E31" t="s">
-        <v>112</v>
-      </c>
-      <c r="F31" t="s">
-        <v>113</v>
-      </c>
-      <c r="G31" t="s">
-        <v>114</v>
-      </c>
-      <c r="H31" s="1">
-        <v>45966</v>
-      </c>
-      <c r="I31" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
+        <v>109</v>
+      </c>
+      <c r="B32" t="s">
+        <v>110</v>
+      </c>
+      <c r="C32">
+        <v>1155</v>
+      </c>
+      <c r="D32" t="s">
+        <v>111</v>
+      </c>
+      <c r="E32" t="s">
+        <v>112</v>
+      </c>
+      <c r="F32" t="s">
+        <v>113</v>
+      </c>
+      <c r="G32" t="s">
+        <v>114</v>
+      </c>
+      <c r="H32" s="1">
+        <v>45966</v>
+      </c>
+      <c r="I32" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>115</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B33" t="s">
         <v>116</v>
       </c>
-      <c r="C32">
+      <c r="C33">
         <v>2056</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D33" t="s">
         <v>55</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E33" t="s">
         <v>88</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F33" t="s">
         <v>42</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G33" t="s">
         <v>117</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H33" s="1">
         <v>45919</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C33">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="C34">
         <v>1547</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D34" t="s">
         <v>118</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E34" t="s">
         <v>119</v>
-      </c>
-      <c r="F33" t="s">
-        <v>120</v>
-      </c>
-      <c r="G33" t="s">
-        <v>121</v>
-      </c>
-      <c r="H33" s="1">
-        <v>45981</v>
-      </c>
-      <c r="I33" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>122</v>
-      </c>
-      <c r="B34" t="s">
-        <v>123</v>
-      </c>
-      <c r="C34">
-        <v>1671</v>
-      </c>
-      <c r="D34" t="s">
-        <v>124</v>
-      </c>
-      <c r="E34" t="s">
-        <v>125</v>
       </c>
       <c r="F34" t="s">
         <v>120</v>
       </c>
       <c r="G34" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="H34" s="1">
-        <v>46072</v>
+        <v>45981</v>
       </c>
       <c r="I34" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B35" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="C35">
-        <v>1662</v>
+        <v>1671</v>
       </c>
       <c r="D35" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="E35" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="F35" t="s">
         <v>120</v>
       </c>
       <c r="G35" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="H35" s="1">
-        <v>45964</v>
+        <v>46072</v>
+      </c>
+      <c r="I35" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>132</v>
+        <v>127</v>
+      </c>
+      <c r="B36" t="s">
+        <v>128</v>
       </c>
       <c r="C36">
-        <v>2055</v>
+        <v>1662</v>
       </c>
       <c r="D36" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="E36" t="s">
-        <v>35</v>
+        <v>130</v>
       </c>
       <c r="F36" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="G36" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="H36" s="1">
-        <v>45931</v>
+        <v>45964</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C37">
-        <v>1888</v>
+        <v>2055</v>
       </c>
       <c r="D37" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E37" t="s">
-        <v>112</v>
+        <v>35</v>
       </c>
       <c r="F37" t="s">
-        <v>63</v>
+        <v>134</v>
       </c>
       <c r="G37" t="s">
-        <v>64</v>
+        <v>135</v>
       </c>
       <c r="H37" s="1">
-        <v>46057</v>
-      </c>
-      <c r="I37" t="s">
-        <v>20</v>
+        <v>45931</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C38">
-        <v>1846</v>
+        <v>1888</v>
       </c>
       <c r="D38" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E38" t="s">
-        <v>140</v>
+        <v>112</v>
       </c>
       <c r="F38" t="s">
         <v>63</v>
@@ -2303,105 +2306,102 @@
         <v>64</v>
       </c>
       <c r="H38" s="1">
-        <v>45983</v>
+        <v>46057</v>
       </c>
       <c r="I38" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C39">
-        <v>1710</v>
+        <v>1846</v>
       </c>
       <c r="D39" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E39" t="s">
-        <v>62</v>
+        <v>140</v>
       </c>
       <c r="F39" t="s">
         <v>63</v>
       </c>
       <c r="G39" t="s">
-        <v>143</v>
+        <v>64</v>
       </c>
       <c r="H39" s="1">
-        <v>45982</v>
+        <v>45983</v>
       </c>
       <c r="I39" t="s">
-        <v>47</v>
+        <v>27</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C40">
-        <v>1897</v>
+        <v>1710</v>
       </c>
       <c r="D40" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E40" t="s">
-        <v>17</v>
+        <v>62</v>
       </c>
       <c r="F40" t="s">
         <v>63</v>
       </c>
       <c r="G40" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="H40" s="1">
-        <v>46015</v>
+        <v>45982</v>
       </c>
       <c r="I40" t="s">
-        <v>20</v>
+        <v>47</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C41">
-        <v>1066</v>
+        <v>1897</v>
       </c>
       <c r="D41" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="E41" t="s">
-        <v>149</v>
+        <v>17</v>
       </c>
       <c r="F41" t="s">
-        <v>150</v>
+        <v>63</v>
       </c>
       <c r="G41" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="H41" s="1">
-        <v>46019</v>
+        <v>46015</v>
       </c>
       <c r="I41" t="s">
-        <v>68</v>
+        <v>20</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>152</v>
-      </c>
-      <c r="B42" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="C42">
-        <v>1072</v>
+        <v>1066</v>
       </c>
       <c r="D42" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="E42" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="F42" t="s">
         <v>150</v>
@@ -2410,27 +2410,27 @@
         <v>151</v>
       </c>
       <c r="H42" s="1">
-        <v>46056</v>
+        <v>46019</v>
       </c>
       <c r="I42" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B43" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C43">
-        <v>1006</v>
+        <v>1072</v>
       </c>
       <c r="D43" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="E43" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="F43" t="s">
         <v>150</v>
@@ -2439,7 +2439,7 @@
         <v>151</v>
       </c>
       <c r="H43" s="1">
-        <v>46033</v>
+        <v>46056</v>
       </c>
       <c r="I43" t="s">
         <v>47</v>
@@ -2447,13 +2447,19 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>160</v>
+        <v>156</v>
+      </c>
+      <c r="B44" t="s">
+        <v>157</v>
+      </c>
+      <c r="C44">
+        <v>1006</v>
       </c>
       <c r="D44" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E44" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="F44" t="s">
         <v>150</v>
@@ -2462,21 +2468,21 @@
         <v>151</v>
       </c>
       <c r="H44" s="1">
-        <v>45939</v>
+        <v>46033</v>
       </c>
       <c r="I44" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D45" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E45" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="F45" t="s">
         <v>150</v>
@@ -2485,142 +2491,136 @@
         <v>151</v>
       </c>
       <c r="H45" s="1">
-        <v>45894</v>
+        <v>45939</v>
       </c>
       <c r="I45" t="s">
-        <v>91</v>
+        <v>53</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D46" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E46" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="F46" t="s">
-        <v>168</v>
+        <v>150</v>
       </c>
       <c r="G46" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="H46" s="1">
-        <v>45873</v>
+        <v>45894</v>
+      </c>
+      <c r="I46" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="D47" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="E47" t="s">
-        <v>17</v>
+        <v>167</v>
       </c>
       <c r="F47" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="G47" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="H47" s="1">
-        <v>46062</v>
+        <v>45873</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>174</v>
-      </c>
-      <c r="B48" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="D48" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="E48" t="s">
-        <v>112</v>
+        <v>17</v>
       </c>
       <c r="F48" t="s">
-        <v>42</v>
+        <v>172</v>
       </c>
       <c r="G48" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="H48" s="1">
-        <v>45871</v>
-      </c>
-      <c r="I48" t="s">
-        <v>53</v>
+        <v>46062</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
+        <v>174</v>
+      </c>
+      <c r="B49" t="s">
+        <v>175</v>
+      </c>
+      <c r="D49" t="s">
+        <v>176</v>
+      </c>
+      <c r="E49" t="s">
+        <v>112</v>
+      </c>
+      <c r="F49" t="s">
+        <v>42</v>
+      </c>
+      <c r="G49" t="s">
+        <v>177</v>
+      </c>
+      <c r="H49" s="1">
+        <v>45871</v>
+      </c>
+      <c r="I49" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
         <v>178</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B50" t="s">
         <v>179</v>
       </c>
-      <c r="C49">
+      <c r="C50">
         <v>1282</v>
       </c>
-      <c r="D49" t="s">
+      <c r="D50" t="s">
         <v>180</v>
       </c>
-      <c r="E49" t="s">
+      <c r="E50" t="s">
         <v>140</v>
       </c>
-      <c r="F49" t="s">
+      <c r="F50" t="s">
         <v>181</v>
       </c>
-      <c r="G49" t="s">
+      <c r="G50" t="s">
         <v>182</v>
       </c>
-      <c r="H49" s="1">
+      <c r="H50" s="1">
         <v>45931</v>
       </c>
-      <c r="I49" t="s">
+      <c r="I50" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B50" t="s">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B51" t="s">
         <v>183</v>
       </c>
-      <c r="E50" t="s">
+      <c r="E51" t="s">
         <v>184</v>
-      </c>
-      <c r="F50" t="s">
-        <v>185</v>
-      </c>
-      <c r="G50" t="s">
-        <v>186</v>
-      </c>
-      <c r="H50" s="1">
-        <v>45955</v>
-      </c>
-      <c r="I50" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>187</v>
-      </c>
-      <c r="B51" t="s">
-        <v>188</v>
-      </c>
-      <c r="C51">
-        <v>2550</v>
-      </c>
-      <c r="D51" t="s">
-        <v>189</v>
-      </c>
-      <c r="E51" t="s">
-        <v>190</v>
       </c>
       <c r="F51" t="s">
         <v>185</v>
@@ -2629,53 +2629,53 @@
         <v>186</v>
       </c>
       <c r="H51" s="1">
-        <v>45882</v>
+        <v>45955</v>
+      </c>
+      <c r="I51" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B52" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C52">
-        <v>1428</v>
+        <v>2550</v>
       </c>
       <c r="D52" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="E52" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F52" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="G52" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="H52" s="1">
-        <v>46079</v>
-      </c>
-      <c r="I52" t="s">
-        <v>103</v>
+        <v>45882</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>197</v>
-      </c>
-      <c r="B53" s="1">
-        <v>2023695</v>
+        <v>191</v>
+      </c>
+      <c r="B53" t="s">
+        <v>192</v>
       </c>
       <c r="C53">
-        <v>2257</v>
+        <v>1428</v>
       </c>
       <c r="D53" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="E53" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="F53" t="s">
         <v>195</v>
@@ -2684,24 +2684,27 @@
         <v>196</v>
       </c>
       <c r="H53" s="1">
-        <v>45928</v>
+        <v>46079</v>
+      </c>
+      <c r="I53" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>200</v>
-      </c>
-      <c r="B54" t="s">
-        <v>201</v>
+        <v>197</v>
+      </c>
+      <c r="B54" s="1">
+        <v>2023695</v>
       </c>
       <c r="C54">
-        <v>1415</v>
+        <v>2257</v>
       </c>
       <c r="D54" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="E54" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="F54" t="s">
         <v>195</v>
@@ -2710,10 +2713,65 @@
         <v>196</v>
       </c>
       <c r="H54" s="1">
+        <v>45928</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>200</v>
+      </c>
+      <c r="B55" t="s">
+        <v>201</v>
+      </c>
+      <c r="C55">
+        <v>1415</v>
+      </c>
+      <c r="D55" t="s">
+        <v>202</v>
+      </c>
+      <c r="E55" t="s">
+        <v>203</v>
+      </c>
+      <c r="F55" t="s">
+        <v>195</v>
+      </c>
+      <c r="G55" t="s">
+        <v>196</v>
+      </c>
+      <c r="H55" s="1">
         <v>45921</v>
       </c>
-      <c r="I54" t="s">
+      <c r="I55" t="s">
         <v>103</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>204</v>
+      </c>
+      <c r="B56" t="s">
+        <v>0</v>
+      </c>
+      <c r="C56" t="s">
+        <v>1</v>
+      </c>
+      <c r="D56" t="s">
+        <v>2</v>
+      </c>
+      <c r="E56" t="s">
+        <v>3</v>
+      </c>
+      <c r="F56" t="s">
+        <v>4</v>
+      </c>
+      <c r="G56" t="s">
+        <v>5</v>
+      </c>
+      <c r="H56" t="s">
+        <v>6</v>
+      </c>
+      <c r="I56" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>